<commit_message>
Sample med prompt responses
</commit_message>
<xml_diff>
--- a/TrainingEpidolex.xlsx
+++ b/TrainingEpidolex.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mepragel/Documents/CMPSC 488/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mepragel/Documents/CMPSC 488/Smart-Glass-Medical-Assistant/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CBE13E3-A645-534B-947B-185E4AFCCEF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8FB2DC3-2BAE-DC40-B83E-FEA171C9A05C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12800" yWindow="2680" windowWidth="28040" windowHeight="17440" xr2:uid="{9F4A9061-966E-7847-9CFB-ECFE57086142}"/>
+    <workbookView xWindow="8500" yWindow="2380" windowWidth="28040" windowHeight="17440" xr2:uid="{9F4A9061-966E-7847-9CFB-ECFE57086142}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -66,7 +66,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -75,16 +75,23 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
+      <b/>
+      <sz val="22"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="22"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
     <font>
-      <b/>
-      <sz val="12"/>
+      <sz val="22"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -108,10 +115,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -446,44 +460,96 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64232C2C-9368-1E4B-A7CF-496F0BA4AF07}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="53.83203125" customWidth="1"/>
-    <col min="2" max="2" width="38.33203125" customWidth="1"/>
+    <col min="1" max="1" width="78" customWidth="1"/>
+    <col min="2" max="2" width="57.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:2" ht="30" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:2" ht="59" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+    <row r="3" spans="1:2" ht="60" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+    <row r="4" spans="1:2" ht="60" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="3" t="s">
         <v>7</v>
       </c>
+    </row>
+    <row r="5" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+    </row>
+    <row r="6" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A6" s="3"/>
+      <c r="B6" s="3"/>
+    </row>
+    <row r="7" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+    </row>
+    <row r="8" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A8" s="3"/>
+      <c r="B8" s="3"/>
+    </row>
+    <row r="9" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A9" s="3"/>
+      <c r="B9" s="3"/>
+    </row>
+    <row r="10" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A10" s="3"/>
+      <c r="B10" s="3"/>
+    </row>
+    <row r="11" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A11" s="3"/>
+      <c r="B11" s="3"/>
+    </row>
+    <row r="12" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+    </row>
+    <row r="13" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A13" s="3"/>
+      <c r="B13" s="3"/>
+    </row>
+    <row r="14" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A14" s="3"/>
+      <c r="B14" s="3"/>
+    </row>
+    <row r="15" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A15" s="3"/>
+      <c r="B15" s="3"/>
+    </row>
+    <row r="16" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A16" s="3"/>
+      <c r="B16" s="3"/>
+    </row>
+    <row r="17" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A17" s="3"/>
+      <c r="B17" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>